<commit_message>
atualizacao das saidas dos testes de alocacao
</commit_message>
<xml_diff>
--- a/alocacao/saidas/resumo_custos.xlsx
+++ b/alocacao/saidas/resumo_custos.xlsx
@@ -413,17 +413,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
     <col width="19" customWidth="1" min="2" max="2"/>
-    <col width="9" customWidth="1" min="3" max="3"/>
-    <col width="25" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="9" customWidth="1" min="6" max="6"/>
-    <col width="89" customWidth="1" min="7" max="7"/>
-    <col width="92" customWidth="1" min="8" max="8"/>
+    <col width="33" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="89" customWidth="1" min="8" max="8"/>
+    <col width="92" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -439,30 +440,35 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>Pico de Abastecimento (Max/Dia)</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Custo Modelo Exato (M1)</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Custo Heurística</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Gap (%)</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Caminho da Entrada</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Pasta de Saída</t>
         </is>
@@ -475,28 +481,31 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3315</v>
-      </c>
-      <c r="C2" t="inlineStr">
+        <v>43418</v>
+      </c>
+      <c r="C2" t="n">
+        <v>498</v>
+      </c>
+      <c r="D2" t="inlineStr">
         <is>
           <t>Sucesso</t>
         </is>
       </c>
-      <c r="D2" t="n">
-        <v>2223257.660377</v>
-      </c>
       <c r="E2" t="n">
-        <v>2467920.5028</v>
+        <v>2223257.66</v>
       </c>
       <c r="F2" t="n">
+        <v>2467920.5</v>
+      </c>
+      <c r="G2" t="n">
         <v>11</v>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas\00.csv</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas\alocacao_00</t>
         </is>
@@ -509,28 +518,31 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>3315</v>
-      </c>
-      <c r="C3" t="inlineStr">
+        <v>47702</v>
+      </c>
+      <c r="C3" t="n">
+        <v>230</v>
+      </c>
+      <c r="D3" t="inlineStr">
         <is>
           <t>Sucesso</t>
         </is>
       </c>
-      <c r="D3" t="n">
-        <v>2447547.159803</v>
-      </c>
       <c r="E3" t="n">
-        <v>2492096.5648</v>
+        <v>2447547.16</v>
       </c>
       <c r="F3" t="n">
+        <v>2492096.56</v>
+      </c>
+      <c r="G3" t="n">
         <v>1.82</v>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas\01w24.csv</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas\alocacao_01w24</t>
         </is>
@@ -543,28 +555,31 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>3315</v>
-      </c>
-      <c r="C4" t="inlineStr">
+        <v>43430</v>
+      </c>
+      <c r="C4" t="n">
+        <v>259</v>
+      </c>
+      <c r="D4" t="inlineStr">
         <is>
           <t>Sucesso</t>
         </is>
       </c>
-      <c r="D4" t="n">
-        <v>2228923.934551001</v>
-      </c>
       <c r="E4" t="n">
-        <v>2261986.8442</v>
+        <v>2228923.93</v>
       </c>
       <c r="F4" t="n">
+        <v>2261986.84</v>
+      </c>
+      <c r="G4" t="n">
         <v>1.48</v>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas\10wLim.csv</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas\alocacao_10wLim</t>
         </is>
@@ -577,28 +592,31 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>3315</v>
-      </c>
-      <c r="C5" t="inlineStr">
+        <v>45263</v>
+      </c>
+      <c r="C5" t="n">
+        <v>202</v>
+      </c>
+      <c r="D5" t="inlineStr">
         <is>
           <t>Sucesso</t>
         </is>
       </c>
-      <c r="D5" t="n">
-        <v>2338453.495928</v>
-      </c>
       <c r="E5" t="n">
-        <v>2379435.4346</v>
+        <v>2338453.5</v>
       </c>
       <c r="F5" t="n">
+        <v>2379435.43</v>
+      </c>
+      <c r="G5" t="n">
         <v>1.75</v>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas\5072h.csv</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas\alocacao_5072h</t>
         </is>
@@ -611,28 +629,31 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>3315</v>
-      </c>
-      <c r="C6" t="inlineStr">
+        <v>47076</v>
+      </c>
+      <c r="C6" t="n">
+        <v>212</v>
+      </c>
+      <c r="D6" t="inlineStr">
         <is>
           <t>Sucesso</t>
         </is>
       </c>
-      <c r="D6" t="n">
-        <v>2409050.893031</v>
-      </c>
       <c r="E6" t="n">
-        <v>2450491.1585</v>
+        <v>2409050.89</v>
       </c>
       <c r="F6" t="n">
+        <v>2450491.16</v>
+      </c>
+      <c r="G6" t="n">
         <v>1.72</v>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas\50wLim.csv</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas\alocacao_50wLim</t>
         </is>
@@ -645,28 +666,31 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>3315</v>
-      </c>
-      <c r="C7" t="inlineStr">
+        <v>49421</v>
+      </c>
+      <c r="C7" t="n">
+        <v>227</v>
+      </c>
+      <c r="D7" t="inlineStr">
         <is>
           <t>Sucesso</t>
         </is>
       </c>
-      <c r="D7" t="n">
-        <v>2537623.539127</v>
-      </c>
       <c r="E7" t="n">
-        <v>2591364.9433</v>
+        <v>2537623.54</v>
       </c>
       <c r="F7" t="n">
+        <v>2591364.94</v>
+      </c>
+      <c r="G7" t="n">
         <v>2.12</v>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas\75w00.csv</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas\alocacao_75w00</t>
         </is>

</xml_diff>

<commit_message>
Resultados teste de alocacao
</commit_message>
<xml_diff>
--- a/alocacao/saidas/resumo_custos.xlsx
+++ b/alocacao/saidas/resumo_custos.xlsx
@@ -46,8 +46,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,18 +417,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:K9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="19" customWidth="1" min="1" max="1"/>
-    <col width="19" customWidth="1" min="2" max="2"/>
-    <col width="33" customWidth="1" min="3" max="3"/>
-    <col width="9" customWidth="1" min="4" max="4"/>
-    <col width="25" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="9" customWidth="1" min="7" max="7"/>
-    <col width="89" customWidth="1" min="8" max="8"/>
-    <col width="92" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="19" customWidth="1" min="7" max="7"/>
+    <col width="27" customWidth="1" min="8" max="8"/>
+    <col width="19" customWidth="1" min="9" max="9"/>
+    <col width="92" customWidth="1" min="10" max="10"/>
+    <col width="95" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -455,35 +461,45 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
+          <t>Custo Modelo Anual (M2)</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
           <t>Custo Heurística</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Gap (%)</t>
-        </is>
-      </c>
       <c r="H1" t="inlineStr">
         <is>
+          <t>Gap Heurística vs M1 (%)</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Gap M2 vs M1 (%)</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
           <t>Caminho da Entrada</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Pasta de Saída</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>00</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="B2" s="2" t="n">
         <v>43418</v>
       </c>
-      <c r="C2" t="n">
+      <c r="C2" s="2" t="n">
         <v>498</v>
       </c>
       <c r="D2" t="inlineStr">
@@ -491,36 +507,42 @@
           <t>Sucesso</t>
         </is>
       </c>
-      <c r="E2" t="n">
+      <c r="E2" s="3" t="n">
         <v>2223257.66</v>
       </c>
-      <c r="F2" t="n">
+      <c r="F2" s="3" t="n">
+        <v>2223489.44</v>
+      </c>
+      <c r="G2" s="3" t="n">
         <v>2467920.5</v>
       </c>
-      <c r="G2" t="n">
+      <c r="H2" s="4" t="n">
         <v>11</v>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" s="4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="J2" t="inlineStr">
         <is>
           <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas\00.csv</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas\alocacao_00</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>01w24</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="B3" s="2" t="n">
         <v>47702</v>
       </c>
-      <c r="C3" t="n">
+      <c r="C3" s="2" t="n">
         <v>230</v>
       </c>
       <c r="D3" t="inlineStr">
@@ -528,36 +550,42 @@
           <t>Sucesso</t>
         </is>
       </c>
-      <c r="E3" t="n">
+      <c r="E3" s="3" t="n">
         <v>2447547.16</v>
       </c>
-      <c r="F3" t="n">
+      <c r="F3" s="3" t="n">
+        <v>2447547.16</v>
+      </c>
+      <c r="G3" s="3" t="n">
         <v>2492096.56</v>
       </c>
-      <c r="G3" t="n">
+      <c r="H3" s="4" t="n">
         <v>1.82</v>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="I3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" t="inlineStr">
         <is>
           <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas\01w24.csv</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas\alocacao_01w24</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>10wLim</t>
         </is>
       </c>
-      <c r="B4" t="n">
+      <c r="B4" s="2" t="n">
         <v>43430</v>
       </c>
-      <c r="C4" t="n">
+      <c r="C4" s="2" t="n">
         <v>259</v>
       </c>
       <c r="D4" t="inlineStr">
@@ -565,36 +593,42 @@
           <t>Sucesso</t>
         </is>
       </c>
-      <c r="E4" t="n">
+      <c r="E4" s="3" t="n">
         <v>2228923.93</v>
       </c>
-      <c r="F4" t="n">
+      <c r="F4" s="3" t="n">
+        <v>2228923.93</v>
+      </c>
+      <c r="G4" s="3" t="n">
         <v>2261986.84</v>
       </c>
-      <c r="G4" t="n">
+      <c r="H4" s="4" t="n">
         <v>1.48</v>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="I4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" t="inlineStr">
         <is>
           <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas\10wLim.csv</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas\alocacao_10wLim</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="1" t="inlineStr">
         <is>
           <t>5072h</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="B5" s="2" t="n">
         <v>45263</v>
       </c>
-      <c r="C5" t="n">
+      <c r="C5" s="2" t="n">
         <v>202</v>
       </c>
       <c r="D5" t="inlineStr">
@@ -602,36 +636,42 @@
           <t>Sucesso</t>
         </is>
       </c>
-      <c r="E5" t="n">
+      <c r="E5" s="3" t="n">
         <v>2338453.5</v>
       </c>
-      <c r="F5" t="n">
+      <c r="F5" s="3" t="n">
+        <v>2338459.2</v>
+      </c>
+      <c r="G5" s="3" t="n">
         <v>2379435.43</v>
       </c>
-      <c r="G5" t="n">
+      <c r="H5" s="4" t="n">
         <v>1.75</v>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="I5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" t="inlineStr">
         <is>
           <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas\5072h.csv</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas\alocacao_5072h</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="1" t="inlineStr">
         <is>
           <t>50wLim</t>
         </is>
       </c>
-      <c r="B6" t="n">
+      <c r="B6" s="2" t="n">
         <v>47076</v>
       </c>
-      <c r="C6" t="n">
+      <c r="C6" s="2" t="n">
         <v>212</v>
       </c>
       <c r="D6" t="inlineStr">
@@ -639,36 +679,42 @@
           <t>Sucesso</t>
         </is>
       </c>
-      <c r="E6" t="n">
+      <c r="E6" s="3" t="n">
         <v>2409050.89</v>
       </c>
-      <c r="F6" t="n">
+      <c r="F6" s="3" t="n">
+        <v>2409057.53</v>
+      </c>
+      <c r="G6" s="3" t="n">
         <v>2450491.16</v>
       </c>
-      <c r="G6" t="n">
+      <c r="H6" s="4" t="n">
         <v>1.72</v>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="I6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" t="inlineStr">
         <is>
           <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas\50wLim.csv</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas\alocacao_50wLim</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="1" t="inlineStr">
         <is>
           <t>75w00</t>
         </is>
       </c>
-      <c r="B7" t="n">
+      <c r="B7" s="2" t="n">
         <v>49421</v>
       </c>
-      <c r="C7" t="n">
+      <c r="C7" s="2" t="n">
         <v>227</v>
       </c>
       <c r="D7" t="inlineStr">
@@ -676,23 +722,115 @@
           <t>Sucesso</t>
         </is>
       </c>
-      <c r="E7" t="n">
+      <c r="E7" s="3" t="n">
         <v>2537623.54</v>
       </c>
-      <c r="F7" t="n">
+      <c r="F7" s="3" t="n">
+        <v>2537623.54</v>
+      </c>
+      <c r="G7" s="3" t="n">
         <v>2591364.94</v>
       </c>
-      <c r="G7" t="n">
+      <c r="H7" s="4" t="n">
         <v>2.12</v>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="I7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" t="inlineStr">
         <is>
           <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas\75w00.csv</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="K7" t="inlineStr">
         <is>
           <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas\alocacao_75w00</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>heu_full</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>43379</v>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>568</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>2244053.44</v>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>2244177.41</v>
+      </c>
+      <c r="G8" s="3" t="n">
+        <v>2583535.61</v>
+      </c>
+      <c r="H8" s="4" t="n">
+        <v>15.13</v>
+      </c>
+      <c r="I8" s="4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas\heu_full.csv</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas\alocacao_heu_full</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>heu_lim</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>43041</v>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>571</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>2226392.05</v>
+      </c>
+      <c r="F9" s="3" t="n">
+        <v>2226520.62</v>
+      </c>
+      <c r="G9" s="3" t="n">
+        <v>2549352.76</v>
+      </c>
+      <c r="H9" s="4" t="n">
+        <v>14.51</v>
+      </c>
+      <c r="I9" s="4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas\heu_lim.csv</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas\alocacao_heu_lim</t>
         </is>
       </c>
     </row>

</xml_diff>